<commit_message>
feat: expand spreadsheet editing and reliable saves
</commit_message>
<xml_diff>
--- a/src/test/fixtures/xlsx/formula_excel.xlsx
+++ b/src/test/fixtures/xlsx/formula_excel.xlsx
@@ -12585,23 +12585,23 @@
         <v/>
       </c>
       <c r="B3">
-        <f>VLOOKUP(A2,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A3,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D3">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A2,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A3,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E3">
-        <f>MATCH(A2,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A3,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F3">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A2,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A3,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G3">
@@ -12635,23 +12635,23 @@
         <v/>
       </c>
       <c r="B4">
-        <f>VLOOKUP(A3,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A4,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D4">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A3,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A4,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E4">
-        <f>MATCH(A3,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A4,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F4">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A3,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A4,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G4">
@@ -12685,23 +12685,23 @@
         <v/>
       </c>
       <c r="B5">
-        <f>VLOOKUP(A4,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A5,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D5">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A4,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A5,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E5">
-        <f>MATCH(A4,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A5,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F5">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A4,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A5,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G5">
@@ -12735,23 +12735,23 @@
         <v/>
       </c>
       <c r="B6">
-        <f>VLOOKUP(A5,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A6,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C6">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D6">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A5,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A6,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E6">
-        <f>MATCH(A5,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A6,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F6">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A5,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A6,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G6">
@@ -12785,23 +12785,23 @@
         <v/>
       </c>
       <c r="B7">
-        <f>VLOOKUP(A6,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A7,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C7">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D7">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A6,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A7,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E7">
-        <f>MATCH(A6,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A7,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F7">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A6,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A7,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G7">
@@ -12835,23 +12835,23 @@
         <v/>
       </c>
       <c r="B8">
-        <f>VLOOKUP(A7,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A8,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D8">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A7,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A8,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E8">
-        <f>MATCH(A7,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A8,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F8">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A7,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A8,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G8">
@@ -12885,23 +12885,23 @@
         <v/>
       </c>
       <c r="B9">
-        <f>VLOOKUP(A8,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A9,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D9">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A8,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A9,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E9">
-        <f>MATCH(A8,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A9,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F9">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A8,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A9,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G9">
@@ -12935,23 +12935,23 @@
         <v/>
       </c>
       <c r="B10">
-        <f>VLOOKUP(A9,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A10,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D10">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A9,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A10,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E10">
-        <f>MATCH(A9,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A10,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F10">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A9,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A10,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G10">
@@ -12985,23 +12985,23 @@
         <v/>
       </c>
       <c r="B11">
-        <f>VLOOKUP(A10,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A11,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D11">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A10,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A11,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E11">
-        <f>MATCH(A10,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A11,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F11">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A10,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A11,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G11">
@@ -13035,23 +13035,23 @@
         <v/>
       </c>
       <c r="B12">
-        <f>VLOOKUP(A11,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A12,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D12">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A11,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A12,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E12">
-        <f>MATCH(A11,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A12,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F12">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A11,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A12,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G12">
@@ -13085,23 +13085,23 @@
         <v/>
       </c>
       <c r="B13">
-        <f>VLOOKUP(A12,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A13,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D13">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A12,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A13,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E13">
-        <f>MATCH(A12,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A13,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F13">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A12,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A13,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G13">
@@ -13135,23 +13135,23 @@
         <v/>
       </c>
       <c r="B14">
-        <f>VLOOKUP(A13,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A14,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C14">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D14">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A13,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A14,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E14">
-        <f>MATCH(A13,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A14,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F14">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A13,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A14,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G14">
@@ -13185,23 +13185,23 @@
         <v/>
       </c>
       <c r="B15">
-        <f>VLOOKUP(A14,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A15,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C15">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D15">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A14,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A15,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E15">
-        <f>MATCH(A14,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A15,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F15">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A14,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A15,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G15">
@@ -13235,23 +13235,23 @@
         <v/>
       </c>
       <c r="B16">
-        <f>VLOOKUP(A15,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A16,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D16">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A15,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A16,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E16">
-        <f>MATCH(A15,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A16,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F16">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A15,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A16,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G16">
@@ -13285,23 +13285,23 @@
         <v/>
       </c>
       <c r="B17">
-        <f>VLOOKUP(A16,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A17,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D17">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A16,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A17,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E17">
-        <f>MATCH(A16,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A17,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F17">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A16,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A17,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G17">
@@ -13335,23 +13335,23 @@
         <v/>
       </c>
       <c r="B18">
-        <f>VLOOKUP(A17,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A18,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D18">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A17,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A18,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E18">
-        <f>MATCH(A17,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A18,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F18">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A17,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A18,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G18">
@@ -13385,23 +13385,23 @@
         <v/>
       </c>
       <c r="B19">
-        <f>VLOOKUP(A18,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A19,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D19">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A18,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A19,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E19">
-        <f>MATCH(A18,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A19,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F19">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A18,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A19,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G19">
@@ -13435,23 +13435,23 @@
         <v/>
       </c>
       <c r="B20">
-        <f>VLOOKUP(A19,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A20,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D20">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A19,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A20,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E20">
-        <f>MATCH(A19,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A20,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F20">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A19,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A20,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G20">
@@ -13485,23 +13485,23 @@
         <v/>
       </c>
       <c r="B21">
-        <f>VLOOKUP(A20,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A21,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D21">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A20,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A21,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E21">
-        <f>MATCH(A20,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A21,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F21">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A20,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A21,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G21">
@@ -13535,23 +13535,23 @@
         <v/>
       </c>
       <c r="B22">
-        <f>VLOOKUP(A21,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A22,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D22">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A21,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A22,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E22">
-        <f>MATCH(A21,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A22,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F22">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A21,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A22,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G22">
@@ -13585,23 +13585,23 @@
         <v/>
       </c>
       <c r="B23">
-        <f>VLOOKUP(A22,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A23,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D23">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A22,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A23,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E23">
-        <f>MATCH(A22,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A23,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F23">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A22,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A23,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G23">
@@ -13635,23 +13635,23 @@
         <v/>
       </c>
       <c r="B24">
-        <f>VLOOKUP(A23,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A24,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D24">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A23,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A24,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E24">
-        <f>MATCH(A23,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A24,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F24">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A23,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A24,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G24">
@@ -13685,23 +13685,23 @@
         <v/>
       </c>
       <c r="B25">
-        <f>VLOOKUP(A24,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A25,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D25">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A24,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A25,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E25">
-        <f>MATCH(A24,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A25,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F25">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A24,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A25,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G25">
@@ -13735,23 +13735,23 @@
         <v/>
       </c>
       <c r="B26">
-        <f>VLOOKUP(A25,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A26,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C26">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D26">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A25,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A26,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E26">
-        <f>MATCH(A25,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A26,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F26">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A25,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A26,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G26">
@@ -13785,23 +13785,23 @@
         <v/>
       </c>
       <c r="B27">
-        <f>VLOOKUP(A26,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A27,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C27">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D27">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A26,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A27,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E27">
-        <f>MATCH(A26,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A27,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F27">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A26,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A27,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G27">
@@ -13835,23 +13835,23 @@
         <v/>
       </c>
       <c r="B28">
-        <f>VLOOKUP(A27,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A28,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C28">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D28">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A27,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A28,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E28">
-        <f>MATCH(A27,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A28,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F28">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A27,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A28,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G28">
@@ -13885,23 +13885,23 @@
         <v/>
       </c>
       <c r="B29">
-        <f>VLOOKUP(A28,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A29,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C29">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D29">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A28,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A29,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E29">
-        <f>MATCH(A28,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A29,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F29">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A28,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A29,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G29">
@@ -13935,23 +13935,23 @@
         <v/>
       </c>
       <c r="B30">
-        <f>VLOOKUP(A29,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A30,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C30">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D30">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A29,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A30,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E30">
-        <f>MATCH(A29,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A30,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F30">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A29,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A30,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G30">
@@ -13985,23 +13985,23 @@
         <v/>
       </c>
       <c r="B31">
-        <f>VLOOKUP(A30,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A31,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C31">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D31">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A30,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A31,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E31">
-        <f>MATCH(A30,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A31,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F31">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A30,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A31,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G31">
@@ -14035,23 +14035,23 @@
         <v/>
       </c>
       <c r="B32">
-        <f>VLOOKUP(A31,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A32,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C32">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D32">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A31,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A32,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E32">
-        <f>MATCH(A31,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A32,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F32">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A31,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A32,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G32">
@@ -14085,23 +14085,23 @@
         <v/>
       </c>
       <c r="B33">
-        <f>VLOOKUP(A32,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A33,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C33">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D33">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A32,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A33,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E33">
-        <f>MATCH(A32,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A33,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F33">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A32,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A33,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G33">
@@ -14135,23 +14135,23 @@
         <v/>
       </c>
       <c r="B34">
-        <f>VLOOKUP(A33,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A34,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C34">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D34">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A33,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A34,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E34">
-        <f>MATCH(A33,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A34,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F34">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A33,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A34,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G34">
@@ -14185,23 +14185,23 @@
         <v/>
       </c>
       <c r="B35">
-        <f>VLOOKUP(A34,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A35,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C35">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D35">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A34,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A35,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E35">
-        <f>MATCH(A34,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A35,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F35">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A34,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A35,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G35">
@@ -14235,23 +14235,23 @@
         <v/>
       </c>
       <c r="B36">
-        <f>VLOOKUP(A35,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A36,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C36">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D36">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A35,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A36,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E36">
-        <f>MATCH(A35,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A36,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F36">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A35,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A36,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G36">
@@ -14285,23 +14285,23 @@
         <v/>
       </c>
       <c r="B37">
-        <f>VLOOKUP(A36,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A37,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C37">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D37">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A36,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A37,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E37">
-        <f>MATCH(A36,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A37,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F37">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A36,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A37,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G37">
@@ -14335,23 +14335,23 @@
         <v/>
       </c>
       <c r="B38">
-        <f>VLOOKUP(A37,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A38,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C38">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D38">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A37,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A38,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E38">
-        <f>MATCH(A37,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A38,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F38">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A37,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A38,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G38">
@@ -14385,23 +14385,23 @@
         <v/>
       </c>
       <c r="B39">
-        <f>VLOOKUP(A38,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A39,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C39">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D39">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A38,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A39,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E39">
-        <f>MATCH(A38,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A39,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F39">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A38,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A39,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G39">
@@ -14435,23 +14435,23 @@
         <v/>
       </c>
       <c r="B40">
-        <f>VLOOKUP(A39,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A40,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C40">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D40">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A39,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A40,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E40">
-        <f>MATCH(A39,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A40,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F40">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A39,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A40,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G40">
@@ -14485,23 +14485,23 @@
         <v/>
       </c>
       <c r="B41">
-        <f>VLOOKUP(A40,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A41,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C41">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D41">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A40,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A41,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E41">
-        <f>MATCH(A40,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A41,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F41">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A40,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A41,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G41">
@@ -14535,23 +14535,23 @@
         <v/>
       </c>
       <c r="B42">
-        <f>VLOOKUP(A41,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A42,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C42">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D42">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A41,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A42,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E42">
-        <f>MATCH(A41,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A42,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F42">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A41,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A42,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G42">
@@ -14585,23 +14585,23 @@
         <v/>
       </c>
       <c r="B43">
-        <f>VLOOKUP(A42,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A43,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C43">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D43">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A42,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A43,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E43">
-        <f>MATCH(A42,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A43,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F43">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A42,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A43,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G43">
@@ -14635,23 +14635,23 @@
         <v/>
       </c>
       <c r="B44">
-        <f>VLOOKUP(A43,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A44,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C44">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D44">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A43,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A44,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E44">
-        <f>MATCH(A43,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A44,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F44">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A43,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A44,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G44">
@@ -14685,23 +14685,23 @@
         <v/>
       </c>
       <c r="B45">
-        <f>VLOOKUP(A44,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A45,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C45">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D45">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A44,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A45,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E45">
-        <f>MATCH(A44,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A45,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F45">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A44,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A45,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G45">
@@ -14735,23 +14735,23 @@
         <v/>
       </c>
       <c r="B46">
-        <f>VLOOKUP(A45,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A46,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C46">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D46">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A45,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A46,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E46">
-        <f>MATCH(A45,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A46,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F46">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A45,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A46,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G46">
@@ -14785,23 +14785,23 @@
         <v/>
       </c>
       <c r="B47">
-        <f>VLOOKUP(A46,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A47,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C47">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D47">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A46,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A47,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E47">
-        <f>MATCH(A46,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A47,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F47">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A46,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A47,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G47">
@@ -14835,23 +14835,23 @@
         <v/>
       </c>
       <c r="B48">
-        <f>VLOOKUP(A47,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A48,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C48">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D48">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A47,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A48,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E48">
-        <f>MATCH(A47,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A48,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F48">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A47,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A48,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G48">
@@ -14885,23 +14885,23 @@
         <v/>
       </c>
       <c r="B49">
-        <f>VLOOKUP(A48,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A49,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C49">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D49">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A48,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A49,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E49">
-        <f>MATCH(A48,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A49,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F49">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A48,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A49,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G49">
@@ -14935,23 +14935,23 @@
         <v/>
       </c>
       <c r="B50">
-        <f>VLOOKUP(A49,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A50,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C50">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D50">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A49,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A50,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E50">
-        <f>MATCH(A49,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A50,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F50">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A49,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A50,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G50">
@@ -14985,23 +14985,23 @@
         <v/>
       </c>
       <c r="B51">
-        <f>VLOOKUP(A50,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A51,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C51">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D51">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A50,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A51,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E51">
-        <f>MATCH(A50,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A51,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F51">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A50,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A51,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G51">
@@ -15035,23 +15035,23 @@
         <v/>
       </c>
       <c r="B52">
-        <f>VLOOKUP(A51,Datos!$A$2:$K$51,2,FALSE)</f>
+        <f>VLOOKUP(A52,Datos!$A$2:$K$51,2,FALSE)</f>
         <v/>
       </c>
       <c r="C52">
-        <f>HLOOKUP(MOD(ROW(),3),$N$1:$Q$2,2,FALSE)</f>
+        <f>HLOOKUP(CHOOSE(MOD(ROW()-3,3)+1,"A","B","C"),$O$1:$Q$2,2,FALSE)</f>
         <v/>
       </c>
       <c r="D52">
-        <f>INDEX(Datos!$B$2:$B$51,MATCH(A51,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$B$2:$B$51,MATCH(A52,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="E52">
-        <f>MATCH(A51,Datos!$A$2:$A$51,0)</f>
+        <f>MATCH(A52,Datos!$A$2:$A$51,0)</f>
         <v/>
       </c>
       <c r="F52">
-        <f>INDEX(Datos!$C$2:$C$51,MATCH(A51,Datos!$A$2:$A$51,0))</f>
+        <f>INDEX(Datos!$C$2:$C$51,MATCH(A52,Datos!$A$2:$A$51,0))</f>
         <v/>
       </c>
       <c r="G52">

</xml_diff>